<commit_message>
[Modify][MOS_EXCEL_THI] fix function, login logic, and question scoring
</commit_message>
<xml_diff>
--- a/Data/Excel_Thi/data/9.xlsx
+++ b/Data/Excel_Thi/data/9.xlsx
@@ -1,21 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\MOS360\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell7390\Desktop\File đề test\TEST EXCEL_11P\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7183490-5BCA-44EB-9BB5-80B51E943D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFBFBB58-2F76-4EFB-9331-0B033A19EEDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-30" windowWidth="28920" windowHeight="12960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId3"/>
+  </externalReferences>
   <definedNames>
     <definedName name="Increase">Products!$B$57</definedName>
   </definedNames>
@@ -357,35 +360,35 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="14"/>
       <color theme="4" tint="-0.499984740745262"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="16"/>
       <color theme="4" tint="-0.499984740745262"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
@@ -490,18 +493,55 @@
       </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
+    <c:view3D>
+      <c:rotX val="30"/>
+      <c:rotY val="0"/>
+      <c:depthPercent val="100"/>
+      <c:rAngAx val="0"/>
+    </c:view3D>
+    <c:floor>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:floor>
+    <c:sideWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:sideWall>
+    <c:backWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:backWall>
     <c:plotArea>
       <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
+      <c:pie3DChart>
+        <c:varyColors val="1"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Summary!$B$2</c:f>
+              <c:f>[1]Summary!$B$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -510,19 +550,213 @@
               </c:strCache>
             </c:strRef>
           </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:schemeClr val="lt1"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-D49A-4423-A76A-D6ADFBAD00B2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:schemeClr val="lt1"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-D49A-4423-A76A-D6ADFBAD00B2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:schemeClr val="lt1"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-D49A-4423-A76A-D6ADFBAD00B2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:schemeClr val="lt1"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-D49A-4423-A76A-D6ADFBAD00B2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:schemeClr val="lt1"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-D49A-4423-A76A-D6ADFBAD00B2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:schemeClr val="lt1"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000B-D49A-4423-A76A-D6ADFBAD00B2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="6"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:schemeClr val="lt1"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000D-D49A-4423-A76A-D6ADFBAD00B2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="7"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:schemeClr val="lt1"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000F-D49A-4423-A76A-D6ADFBAD00B2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
           <c:cat>
             <c:strRef>
-              <c:f>Summary!$A$3:$A$10</c:f>
+              <c:f>[1]Summary!$A$3:$A$10</c:f>
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
@@ -554,7 +788,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Summary!$B$3:$B$10</c:f>
+              <c:f>[1]Summary!$B$3:$B$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
@@ -587,7 +821,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D9C7-4E10-9AE6-EE1D2200987C}"/>
+              <c16:uniqueId val="{00000010-D49A-4423-A76A-D6ADFBAD00B2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -598,119 +832,9 @@
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
         </c:dLbls>
-        <c:gapWidth val="219"/>
-        <c:overlap val="-27"/>
-        <c:axId val="242409632"/>
-        <c:axId val="242411592"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="242409632"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="vi-VN"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="242411592"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="242411592"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="vi-VN"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="242409632"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
+      </c:pie3DChart>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -719,6 +843,37 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="vi-VN"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -797,7 +952,7 @@
 </file>
 
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="262">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -854,7 +1009,7 @@
         <a:round/>
       </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:defRPr sz="900" kern="1200"/>
   </cs:chartArea>
   <cs:dataLabel>
     <cs:lnRef idx="0"/>
@@ -905,6 +1060,13 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
   </cs:dataPoint>
   <cs:dataPoint3D>
     <cs:lnRef idx="0"/>
@@ -915,12 +1077,19 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1"/>
+    <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
@@ -958,7 +1127,7 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1"/>
+    <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
@@ -1001,22 +1170,23 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
         </a:schemeClr>
       </a:solidFill>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
             <a:lumMod val="65000"/>
             <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:downBar>
@@ -1121,8 +1291,8 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -1254,19 +1424,20 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -1304,26 +1475,28 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>121920</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:rowOff>83820</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>552450</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>3810</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
+      <xdr:rowOff>112395</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 2">
+        <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1C36E2C1-0467-4751-9101-581876F95346}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -1338,6 +1511,94 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Products"/>
+      <sheetName val="Summary"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1">
+        <row r="2">
+          <cell r="B2" t="str">
+            <v>Quatity</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="A3" t="str">
+            <v>Lab Coats</v>
+          </cell>
+          <cell r="B3">
+            <v>86</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="A4" t="str">
+            <v>Shirts</v>
+          </cell>
+          <cell r="B4">
+            <v>162</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="A5" t="str">
+            <v>Dress</v>
+          </cell>
+          <cell r="B5">
+            <v>55</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="A6" t="str">
+            <v>Uniforms</v>
+          </cell>
+          <cell r="B6">
+            <v>63</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="A7" t="str">
+            <v>Scrub Sets</v>
+          </cell>
+          <cell r="B7">
+            <v>25</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="A8" t="str">
+            <v>Jackets</v>
+          </cell>
+          <cell r="B8">
+            <v>42</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="A9" t="str">
+            <v>Cargo Pants</v>
+          </cell>
+          <cell r="B9">
+            <v>110</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="A10" t="str">
+            <v>Srub Pants</v>
+          </cell>
+          <cell r="B10">
+            <v>44</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1631,18 +1892,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G57"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.5" customWidth="1"/>
-    <col min="2" max="2" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.75" customWidth="1"/>
-    <col min="7" max="7" width="16.875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.77734375" customWidth="1"/>
+    <col min="7" max="7" width="16.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1653,7 +1914,7 @@
       <c r="F1" s="5"/>
       <c r="G1" s="5"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1676,7 +1937,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1696,7 +1957,7 @@
         <v>183.92</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1716,7 +1977,7 @@
         <v>91.96</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1736,7 +1997,7 @@
         <v>252.89</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1756,7 +2017,7 @@
         <v>45.98</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1776,7 +2037,7 @@
         <v>219.8</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1796,7 +2057,7 @@
         <v>141.6</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1816,7 +2077,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1836,7 +2097,7 @@
         <v>23.6</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1856,7 +2117,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1876,7 +2137,7 @@
         <v>70.8</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1896,7 +2157,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -1916,7 +2177,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -1936,7 +2197,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1956,7 +2217,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -1976,7 +2237,7 @@
         <v>220.83</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -1996,7 +2257,7 @@
         <v>259.8</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -2016,7 +2277,7 @@
         <v>259.8</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -2036,7 +2297,7 @@
         <v>194.85</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -2056,7 +2317,7 @@
         <v>157.5</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>24</v>
       </c>
@@ -2076,7 +2337,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -2096,7 +2357,7 @@
         <v>31.5</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -2116,7 +2377,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -2136,7 +2397,7 @@
         <v>134.85</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -2156,7 +2417,7 @@
         <v>179.8</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -2176,7 +2437,7 @@
         <v>71.92</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>25</v>
       </c>
@@ -2196,7 +2457,7 @@
         <v>179.8</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>26</v>
       </c>
@@ -2216,7 +2477,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>30</v>
       </c>
@@ -2236,7 +2497,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>30</v>
       </c>
@@ -2256,7 +2517,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -2276,7 +2537,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -2296,7 +2557,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>33</v>
       </c>
@@ -2316,7 +2577,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>34</v>
       </c>
@@ -2336,7 +2597,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -2356,7 +2617,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>36</v>
       </c>
@@ -2376,7 +2637,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>27</v>
       </c>
@@ -2396,7 +2657,7 @@
         <v>259.89999999999998</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>27</v>
       </c>
@@ -2416,7 +2677,7 @@
         <v>311.88</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>27</v>
       </c>
@@ -2436,7 +2697,7 @@
         <v>233.91</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>27</v>
       </c>
@@ -2456,7 +2717,7 @@
         <v>467.82</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>27</v>
       </c>
@@ -2476,7 +2737,7 @@
         <v>519.79999999999995</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>28</v>
       </c>
@@ -2496,7 +2757,7 @@
         <v>305.82</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>28</v>
       </c>
@@ -2516,7 +2777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>28</v>
       </c>
@@ -2536,7 +2797,7 @@
         <v>152.91999999999999</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>28</v>
       </c>
@@ -2556,7 +2817,7 @@
         <v>135.91999999999999</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>29</v>
       </c>
@@ -2576,7 +2837,7 @@
         <v>79.92</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>29</v>
       </c>
@@ -2596,7 +2857,7 @@
         <v>99.9</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>29</v>
       </c>
@@ -2616,7 +2877,7 @@
         <v>119.88</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>29</v>
       </c>
@@ -2636,7 +2897,7 @@
         <v>153.86000000000001</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>37</v>
       </c>
@@ -2656,7 +2917,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>37</v>
       </c>
@@ -2676,7 +2937,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>37</v>
       </c>
@@ -2696,7 +2957,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>37</v>
       </c>
@@ -2716,7 +2977,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
         <v>80</v>
       </c>
@@ -2740,18 +3001,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.625" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="10.375" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>83</v>
       </c>
@@ -2759,7 +3020,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>92</v>
       </c>
@@ -2767,7 +3028,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>91</v>
       </c>
@@ -2775,7 +3036,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>90</v>
       </c>
@@ -2783,7 +3044,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>89</v>
       </c>
@@ -2791,7 +3052,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>88</v>
       </c>
@@ -2799,7 +3060,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>87</v>
       </c>
@@ -2807,7 +3068,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>86</v>
       </c>
@@ -2815,7 +3076,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>85</v>
       </c>

</xml_diff>